<commit_message>
added vault pki engine function
</commit_message>
<xml_diff>
--- a/Docs/sp800-53b-control-baselines.xlsx
+++ b/Docs/sp800-53b-control-baselines.xlsx
@@ -11594,9 +11594,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>709560</xdr:colOff>
+      <xdr:colOff>708840</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>49320</xdr:rowOff>
+      <xdr:rowOff>48600</xdr:rowOff>
     </xdr:to>
     <xdr:sp>
       <xdr:nvSpPr>
@@ -11606,7 +11606,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="800280" y="889200"/>
-          <a:ext cx="8230320" cy="3865320"/>
+          <a:ext cx="8229600" cy="3864600"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -14459,7 +14459,7 @@
       <c r="F134" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G134" s="9" t="s">
+      <c r="G134" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H134" s="11" t="s">
@@ -14479,7 +14479,7 @@
       <c r="D135" s="13"/>
       <c r="E135" s="14"/>
       <c r="F135" s="14"/>
-      <c r="G135" s="14" t="s">
+      <c r="G135" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H135" s="15" t="s">
@@ -14499,7 +14499,7 @@
       <c r="D136" s="8"/>
       <c r="E136" s="9"/>
       <c r="F136" s="9"/>
-      <c r="G136" s="9" t="s">
+      <c r="G136" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H136" s="11" t="s">
@@ -14567,7 +14567,7 @@
       <c r="D140" s="8"/>
       <c r="E140" s="9"/>
       <c r="F140" s="9"/>
-      <c r="G140" s="9" t="s">
+      <c r="G140" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H140" s="11" t="s">
@@ -14621,7 +14621,7 @@
       <c r="F143" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G143" s="14" t="s">
+      <c r="G143" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H143" s="15" t="s">
@@ -28365,7 +28365,7 @@
       <c r="F884" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G884" s="9" t="s">
+      <c r="G884" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H884" s="11" t="s">
@@ -28385,7 +28385,7 @@
       <c r="D885" s="13"/>
       <c r="E885" s="14"/>
       <c r="F885" s="14"/>
-      <c r="G885" s="14" t="s">
+      <c r="G885" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H885" s="15" t="s">
@@ -28535,7 +28535,7 @@
       <c r="D894" s="8"/>
       <c r="E894" s="9"/>
       <c r="F894" s="9"/>
-      <c r="G894" s="9" t="s">
+      <c r="G894" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H894" s="11" t="s">
@@ -28591,7 +28591,7 @@
       <c r="F897" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="G897" s="14" t="s">
+      <c r="G897" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H897" s="15" t="s">
@@ -28677,7 +28677,7 @@
       <c r="F902" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G902" s="9" t="s">
+      <c r="G902" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H902" s="11" t="s">
@@ -28733,7 +28733,7 @@
       <c r="D905" s="13"/>
       <c r="E905" s="14"/>
       <c r="F905" s="14"/>
-      <c r="G905" s="14" t="s">
+      <c r="G905" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H905" s="15" t="s">
@@ -28753,7 +28753,7 @@
       <c r="D906" s="8"/>
       <c r="E906" s="9"/>
       <c r="F906" s="9"/>
-      <c r="G906" s="9" t="s">
+      <c r="G906" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H906" s="11" t="s">
@@ -28773,7 +28773,7 @@
       <c r="D907" s="13"/>
       <c r="E907" s="14"/>
       <c r="F907" s="14"/>
-      <c r="G907" s="14" t="s">
+      <c r="G907" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H907" s="15" t="s">
@@ -28811,7 +28811,7 @@
       <c r="D909" s="13"/>
       <c r="E909" s="14"/>
       <c r="F909" s="14"/>
-      <c r="G909" s="14" t="s">
+      <c r="G909" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H909" s="15" t="s">
@@ -28831,7 +28831,7 @@
       <c r="D910" s="8"/>
       <c r="E910" s="9"/>
       <c r="F910" s="9"/>
-      <c r="G910" s="9" t="s">
+      <c r="G910" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H910" s="11" t="s">
@@ -29193,7 +29193,7 @@
       <c r="D932" s="8"/>
       <c r="E932" s="9"/>
       <c r="F932" s="9"/>
-      <c r="G932" s="9" t="s">
+      <c r="G932" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H932" s="11" t="s">
@@ -29213,7 +29213,7 @@
       <c r="D933" s="13"/>
       <c r="E933" s="14"/>
       <c r="F933" s="14"/>
-      <c r="G933" s="14" t="s">
+      <c r="G933" s="10" t="s">
         <v>12</v>
       </c>
       <c r="H933" s="15" t="s">

</xml_diff>